<commit_message>
Updated: Added BaseSteps file to invoke initials.
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/ParaBankTestData.xlsx
+++ b/src/test/resources/testdata/ParaBankTestData.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/7717805a7dbae679/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="19" documentId="8_{434B8B22-A38B-4494-A32F-3EB451E65F2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2EBBA786-BFD6-49E6-9BFE-7D6BFB06DC4D}"/>
+  <xr:revisionPtr revIDLastSave="26" documentId="8_{434B8B22-A38B-4494-A32F-3EB451E65F2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D0030F8E-AA75-4A19-8F3C-C7679D93340C}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{1FC8999B-E393-4A79-AD68-370F31348BBB}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{1FC8999B-E393-4A79-AD68-370F31348BBB}"/>
   </bookViews>
   <sheets>
     <sheet name="LoginData" sheetId="1" r:id="rId1"/>
     <sheet name="TransferData" sheetId="2" r:id="rId2"/>
+    <sheet name="AccountOpen" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -35,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="19">
   <si>
     <t>Username</t>
   </si>
@@ -86,13 +87,19 @@
   </si>
   <si>
     <t>Transfer scenario 2</t>
+  </si>
+  <si>
+    <t>Account Open scenario 1</t>
+  </si>
+  <si>
+    <t>Account Open scenario 2</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -112,6 +119,12 @@
       <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -172,10 +185,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -628,4 +637,63 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{91B20FB1-2E48-4A7E-A858-39E65E4ECD66}">
+  <dimension ref="A1:D3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="12.21875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21" customWidth="1"/>
+    <col min="3" max="3" width="21.5546875" customWidth="1"/>
+    <col min="4" max="4" width="30.109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" s="2">
+        <v>22224</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" s="2">
+        <v>56634</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Updated: Added testcase id. handled threads & db pool.
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/ParaBankTestData.xlsx
+++ b/src/test/resources/testdata/ParaBankTestData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/7717805a7dbae679/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="26" documentId="8_{434B8B22-A38B-4494-A32F-3EB451E65F2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D0030F8E-AA75-4A19-8F3C-C7679D93340C}"/>
+  <xr:revisionPtr revIDLastSave="46" documentId="8_{434B8B22-A38B-4494-A32F-3EB451E65F2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A2363C19-DE45-419E-92B3-7D08FB8425E5}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{1FC8999B-E393-4A79-AD68-370F31348BBB}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="27">
   <si>
     <t>Username</t>
   </si>
@@ -93,6 +93,30 @@
   </si>
   <si>
     <t>Account Open scenario 2</t>
+  </si>
+  <si>
+    <t>TestCaseID</t>
+  </si>
+  <si>
+    <t>Login_001</t>
+  </si>
+  <si>
+    <t>Login_002</t>
+  </si>
+  <si>
+    <t>Login_003</t>
+  </si>
+  <si>
+    <t>Transfer_001</t>
+  </si>
+  <si>
+    <t>Transfer_002</t>
+  </si>
+  <si>
+    <t>AcctOpen_001</t>
+  </si>
+  <si>
+    <t>AcctOpen_002</t>
   </si>
 </sst>
 </file>
@@ -185,6 +209,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -504,58 +532,72 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{48F5916A-7DCE-49CD-BE55-229F8C6BB37E}">
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr defaultColWidth="14.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="21" customWidth="1"/>
-    <col min="3" max="3" width="40.21875" customWidth="1"/>
+    <col min="1" max="1" width="17.77734375" customWidth="1"/>
+    <col min="3" max="3" width="21" customWidth="1"/>
+    <col min="4" max="4" width="40.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="C2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="2" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B3" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="C3" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="D3" s="2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B4" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="C4" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="D4" s="2" t="s">
         <v>11</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
@@ -563,132 +605,153 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3D31EE4B-2CAB-4196-B628-9BE71C35705C}">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="12.21875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21" customWidth="1"/>
-    <col min="3" max="3" width="21.5546875" customWidth="1"/>
-    <col min="4" max="4" width="24.5546875" customWidth="1"/>
-    <col min="5" max="5" width="20" customWidth="1"/>
-    <col min="6" max="6" width="30.109375" customWidth="1"/>
+    <col min="1" max="1" width="17.77734375" customWidth="1"/>
+    <col min="2" max="2" width="12.21875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21" customWidth="1"/>
+    <col min="4" max="4" width="21.5546875" customWidth="1"/>
+    <col min="5" max="5" width="24.5546875" customWidth="1"/>
+    <col min="6" max="6" width="20" customWidth="1"/>
+    <col min="7" max="7" width="30.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="C2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="2">
+      <c r="D2" s="2">
         <v>22224</v>
       </c>
-      <c r="D2" s="2">
+      <c r="E2" s="2">
         <v>48309</v>
       </c>
-      <c r="E2" s="2">
+      <c r="F2" s="2">
         <v>10</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="G2" s="2" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B3" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="C3" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="2">
+      <c r="D3" s="2">
         <v>56634</v>
       </c>
-      <c r="D3" s="2">
+      <c r="E3" s="2">
         <v>13344</v>
       </c>
-      <c r="E3" s="2">
+      <c r="F3" s="2">
         <v>25.5</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="G3" s="2" t="s">
         <v>16</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{91B20FB1-2E48-4A7E-A858-39E65E4ECD66}">
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="12.21875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21" customWidth="1"/>
-    <col min="3" max="3" width="21.5546875" customWidth="1"/>
-    <col min="4" max="4" width="30.109375" customWidth="1"/>
+    <col min="1" max="1" width="17.77734375" customWidth="1"/>
+    <col min="2" max="2" width="12.21875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21" customWidth="1"/>
+    <col min="4" max="4" width="21.5546875" customWidth="1"/>
+    <col min="5" max="5" width="30.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="C2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="2">
+      <c r="D2" s="2">
         <v>22224</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="E2" s="2" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B3" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="C3" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="2">
+      <c r="D3" s="2">
         <v>56634</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="E3" s="2" t="s">
         <v>18</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update: App able to login.
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/ParaBankTestData.xlsx
+++ b/src/test/resources/testdata/ParaBankTestData.xlsx
@@ -5,17 +5,18 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/7717805a7dbae679/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mural\OneDrive\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="46" documentId="8_{434B8B22-A38B-4494-A32F-3EB451E65F2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A2363C19-DE45-419E-92B3-7D08FB8425E5}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDFE84DE-C913-4EA5-B98B-893BE3421E03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{1FC8999B-E393-4A79-AD68-370F31348BBB}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{1FC8999B-E393-4A79-AD68-370F31348BBB}"/>
   </bookViews>
   <sheets>
     <sheet name="LoginData" sheetId="1" r:id="rId1"/>
     <sheet name="TransferData" sheetId="2" r:id="rId2"/>
     <sheet name="AccountOpen" sheetId="3" r:id="rId3"/>
+    <sheet name="MobileLoginData" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="27">
   <si>
     <t>Username</t>
   </si>
@@ -209,10 +210,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -759,4 +756,76 @@
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C0264A6-015C-4217-BBBF-1E08A33D6A80}">
+  <dimension ref="A1:D4"/>
+  <sheetFormatPr defaultColWidth="14.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="17.77734375" customWidth="1"/>
+    <col min="3" max="3" width="21" customWidth="1"/>
+    <col min="4" max="4" width="40.21875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>